<commit_message>
feat: Update color scheme and enhance UI components
- Updated color constants in config.py to align with INEGI branding.
- Added new images for sidebar background and logos.
- Implemented user authentication service with JSON user data.
- Created configuration service for managing application settings.
- Developed views for configuration, history, and reports.
- Enhanced login view with password visibility toggle and background image.
- Improved validation view with better error handling and reporting.
- Added functionality to export error reports to Excel.
- Removed temporary Excel file.
</commit_message>
<xml_diff>
--- a/exports/Errores.xlsx
+++ b/exports/Errores.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -494,33 +494,33 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>La respuesta es similar a 'Propios' (score: 0.71)</t>
+          <t>La respuesta es similar a 'Propios'</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>9002</v>
+        <v>9039</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_02O01</t>
+          <t>E_ENAPROCE_05O01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>P2_9X</t>
+          <t>P5_9X</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>La respuesta es similar a 'Propios' (score: 0.68)</t>
+          <t>Longitud mínima no alcanzada</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>9035</v>
+        <v>9002</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -534,27 +534,147 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Texto inválido</t>
+          <t>La respuesta es similar a 'Propios'</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
+        <v>9002</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_04O01</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>P4_9X</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>No especificó otro(as) propietarios(as) o accionistas mayoristas(as)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>9038</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_03O01</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>P3_19X</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>La respuesta es similar a 'Vialidades'</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9038</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_04O01</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>P4_9X</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>No especificó otro(as) propietarios(as) o accionistas mayoristas(as)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_02O01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>P2_9X</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Texto inválido</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_03O01</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>P3_19X</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>La respuesta es similar a 'Vialidades'</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
         <v>9034</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>E_ENAPROCE_02O01</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>P2_9X</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>La respuesta es similar a 'Apoyo gubernamental' (score: 0.68)</t>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>La respuesta es similar a 'Apoyo gubernamental'</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9034</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_04O01</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>P4_9X</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>No especificó otro(as) propietarios(as) o accionistas mayoristas(as)</t>
         </is>
       </c>
     </row>

</xml_diff>